<commit_message>
refactor(delivery-label): clean code, sửa vị trí của các data, add comment
</commit_message>
<xml_diff>
--- a/src/main/resources/template/exportLabel/OB_DeliveryLabelTemplate.xlsx
+++ b/src/main/resources/template/exportLabel/OB_DeliveryLabelTemplate.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Trang_tính1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Template" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -72,6 +72,7 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
       <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
@@ -79,7 +80,8 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10.5"/>
+      <b val="true"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="0"/>
@@ -184,96 +186,88 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -466,7 +460,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B2:K18"/>
+  <dimension ref="B2:J22"/>
   <sheetFormatPr defaultColWidth="9.1484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="1" style="1" width="9.14"/>
@@ -495,174 +489,228 @@
       <c r="I3" s="7"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="8" t="s">
-        <v>1</v>
-      </c>
+      <c r="B4" s="8"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
       <c r="F4" s="9"/>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="5"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="8"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="5"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="8"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="8"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="11"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="5"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="10"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="5"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="12"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="5"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="14"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="16"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="5"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="13"/>
-      <c r="K8" s="13"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
+      <c r="J9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="12"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="6"/>
       <c r="H10" s="6"/>
       <c r="I10" s="7"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="13"/>
+      <c r="J10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="5"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="6"/>
       <c r="H11" s="6"/>
       <c r="I11" s="7"/>
+      <c r="J11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="5"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="17"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="18"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="7"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="5"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
       <c r="I14" s="7"/>
+      <c r="J14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="12"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="19"/>
+      <c r="B15" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="20"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="19"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="20"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="19"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="21"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
       <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="22"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="8"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="5"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="5"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="5"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F14"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B18:F20"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="11" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>